<commit_message>
Publish portable workflow and clean public metadata
</commit_message>
<xml_diff>
--- a/tables/Supplementary_Tables_S1-S7.xlsx
+++ b/tables/Supplementary_Tables_S1-S7.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1a0a8b2bcd474e4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_Polishing" sheetId="2" r:id="Ra32ee37b75fc4726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2_Completeness" sheetId="3" r:id="R7875e85775b94e6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3_Annotation" sheetId="4" r:id="R8231d9d7d0dc4b98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_Functional" sheetId="5" r:id="Rc250b12692aa4f61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_EggNOG_unannot" sheetId="6" r:id="R99e169fe60bf46be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Contig_status" sheetId="7" r:id="R170082f6ad0e4ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_File_inventory" sheetId="8" r:id="Ra5d5f7a5077b4537"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R69275da333f34296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_Polishing" sheetId="2" r:id="R7b705382f8f04379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2_Completeness" sheetId="3" r:id="R3e2702c7e8774d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3_Annotation" sheetId="4" r:id="Rae0cb1c1385d4f9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_Functional" sheetId="5" r:id="R942e7f24fab54344"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_EggNOG_unannot" sheetId="6" r:id="R7298c286a73a4588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Contig_status" sheetId="7" r:id="Rd95db5fa1aa34dae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_File_inventory" sheetId="8" r:id="Rb3614d7ed42240c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8419,7 +8419,7 @@
         <x:v>Internal contig IDs</x:v>
       </x:c>
       <x:c r="F4" s="66" t="str">
-        <x:v>Editor-requested structural backbone; read-depth and repeat-collapse assessment</x:v>
+        <x:v>Structural backbone for read-depth diagnosis and repeat-collapse assessment</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
@@ -8579,7 +8579,7 @@
         <x:v>AC16WH IDs and GenBank protein/contig accessions</x:v>
       </x:c>
       <x:c r="F12" s="66" t="str">
-        <x:v>Complete annotation table requested by the Editor</x:v>
+        <x:v>Complete annotation table for genome-resource reuse</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
@@ -8739,7 +8739,7 @@
         <x:v>Internal contig IDs</x:v>
       </x:c>
       <x:c r="F20" s="66" t="str">
-        <x:v>Removal/trim action report requested by the Editor</x:v>
+        <x:v>Removal and trimming action report</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">

</xml_diff>